<commit_message>
model: add Farmer CBG-Loop Savings sheet to TN model — diesel-vs-CNG mileage (24% gap), FOM high-volume application catch (net -Rs2,300/ha yr1), combined loop ~8% net A2 cut
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pitch/TN-Rice-Mill-Business-Model.xlsx
+++ b/pitch/TN-Rice-Mill-Business-Model.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity — the real risk" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TN Conditions &amp; Sources" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mandi Arrivals (Agmarknet)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Farmer CBG-Loop Savings" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +27,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -104,6 +105,20 @@
       <color rgb="001f5637"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00b7791f"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002f7a4f"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -135,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -174,6 +189,13 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -8275,4 +8297,528 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:H49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2.5" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>TN Paddy Farmer — Diesel→CNG + CBG Loop Savings</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>The paddy-supplier side: how the CBG loop lowers the farmer's cost of production. TN prices, Jul 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>1. DIESEL vs CNG TRACTOR — mileage &amp; fuel cost (TN)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Diesel price (Chennai)</t>
+        </is>
+      </c>
+      <c r="C6" s="38" t="n">
+        <v>99.65000000000001</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>₹/litre</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CNG price (Nagapattinam low)</t>
+        </is>
+      </c>
+      <c r="C7" s="38" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>₹/kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Diesel tractor use (field work)</t>
+        </is>
+      </c>
+      <c r="C8" s="38" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>litres/hour</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Diesel energy</t>
+        </is>
+      </c>
+      <c r="C9" s="38" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>MJ/L; CNG 48 MJ/kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CNG engine efficiency vs diesel</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>spark-ign ~10% less efficient</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>→ CNG use (energy-equivalent)</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="n">
+        <v>4.47</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>kg/hr = 5×38.6/48/0.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Diesel cost / hour</t>
+        </is>
+      </c>
+      <c r="C12" s="39" t="n">
+        <v>498</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>5 L × ₹99.65</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>CNG cost / hour</t>
+        </is>
+      </c>
+      <c r="C13" s="37" t="n">
+        <v>378</v>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>4.47 kg × ₹84.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Fuel saving / hour (mileage gap)</t>
+        </is>
+      </c>
+      <c r="C14" s="37" t="n">
+        <v>120</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>24%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Field hours / acre (paddy)</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>FUEL SAVING / ACRE / SEASON</t>
+        </is>
+      </c>
+      <c r="C16" s="37" t="n">
+        <v>1440</v>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>12 hr × ₹120</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  per hectare</t>
+        </is>
+      </c>
+      <c r="C17" s="35" t="n">
+        <v>3600</v>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>≈ ₹65/qtl at 55 qtl/ha</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>2. BIO-FERTILISER (FOM) — the high-volume application catch</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="n"/>
+      <c r="D19" s="4" t="n"/>
+      <c r="E19" s="4" t="n"/>
+      <c r="F19" s="4" t="n"/>
+      <c r="G19" s="4" t="n"/>
+      <c r="H19" s="4" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Chemical fertiliser cost (paddy)</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>₹/ha</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>FOM replaces (% of fertiliser)</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>→ fertiliser value saved</t>
+        </is>
+      </c>
+      <c r="C22" s="37" t="n">
+        <v>900</v>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>₹/ha</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>FOM volume needed</t>
+        </is>
+      </c>
+      <c r="C23" s="38" t="n">
+        <v>8</v>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>t/ha — FOM ~1-2% N vs urea 46%</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>FOM application cost</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>400</v>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>₹/tonne (load+transport+spread)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>→ application cost of the volume</t>
+        </is>
+      </c>
+      <c r="C25" s="40" t="n">
+        <v>3200</v>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>8 t × ₹400</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>NET FOM (NPK basis, year 1)</t>
+        </is>
+      </c>
+      <c r="C26" s="40" t="n">
+        <v>-2300</v>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>₹900 saved − ₹3,200 to apply</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="41" t="inlineStr">
+        <is>
+          <t>→ THE CATCH: FOM is nutrient-dilute — replacing 15% of fertiliser needs ~8 t/ha of bulky slurry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Spreading that volume costs MORE (₹3,200/ha) than the fertiliser it saves (₹900/ha).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="41" t="inlineStr">
+        <is>
+          <t>→ Turns positive only via: (a) soil-health/organic-carbon yield gain 2-5% over 3-5 yrs (~₹2-4k/ha),</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  (b) near-free FOM from own residue applied close to the CBG plant, (c) PM-PRANAM/FOM support (₹1,500/t).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="41" t="inlineStr">
+        <is>
+          <t>→ HONEST: count FOM as ~break-even year 1 (not a saving); its value is multi-year soil health.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>3. COMBINED CBG LOOP — net effect on paddy cost of production</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="n"/>
+      <c r="D34" s="4" t="n"/>
+      <c r="E34" s="4" t="n"/>
+      <c r="F34" s="4" t="n"/>
+      <c r="G34" s="4" t="n"/>
+      <c r="H34" s="4" t="n"/>
+    </row>
+    <row r="35">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Paddy A2+FL (CACP 2025-26)</t>
+        </is>
+      </c>
+      <c r="C35" s="35" t="n">
+        <v>1579</v>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>₹/qtl</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>+ CNG fuel saving</t>
+        </is>
+      </c>
+      <c r="C36" s="37" t="n">
+        <v>65</v>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>₹3,600/ha ÷ 55 qtl</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>+ Net residue income (straw→CBG)</t>
+        </is>
+      </c>
+      <c r="C37" s="37" t="n">
+        <v>65</v>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>6t×60%×₹1,000/t ÷ 55 qtl</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>+ Net FOM (break-even yr1)</t>
+        </is>
+      </c>
+      <c r="C38" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>long-term soil-health positive, not counted</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39">
+        <f> TOTAL NET BENEFIT</f>
+        <v/>
+      </c>
+      <c r="C39" s="43" t="n">
+        <v>130</v>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>₹/qtl</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40">
+        <f> Net A2+FL improvement</f>
+        <v/>
+      </c>
+      <c r="C40" s="44" t="n">
+        <v>0.082</v>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>8.2% (vs 11.3% before FOM app-cost netted)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="41" t="inlineStr">
+        <is>
+          <t>→ BOTTOM LINE: the CBG loop cuts the TN paddy farmer's net cost of production ~8% —</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  CNG fuel (₹65/qtl) + residue monetisation (₹65/qtl); FOM break-even year 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="41" t="inlineStr">
+        <is>
+          <t>→ Fuel-only diesel→CNG swap is ~3-4%; the loop doubles it via residue income. The bio-fertiliser</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  application cost is the drag that stops FOM adding a third leg on a pure-financial basis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="41" t="inlineStr">
+        <is>
+          <t>→ Lower paddy cost = more competitive paddy supply to the mill (this workbook's feedstock).</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Sources: TN diesel/CNG Jul 2026; PIB CNG-tractor PRID 1697555; FOM/digestate rates+costs (Farmers Weekly,</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>HomeBiogas, biochem lit.); CACP A2+FL. Mileage gap 24% (energy+efficiency adj.). Illustrative — not investment advice.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>